<commit_message>
rubros, sm, acciones, importar csv, registro activos
</commit_message>
<xml_diff>
--- a/partidas.xlsx
+++ b/partidas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuarios\Miliandry\OneDrive\Desktop\PROYECTO_ALMACEN\Pasantias2026-Proyecto-Almacen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d57f09bfa23d157f/Desktop/PROYECTO_ALMACEN/Pasantias2026-Proyecto-Almacen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{299C9AA4-07B9-4E90-B9CB-BA0CEE3DD70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{299C9AA4-07B9-4E90-B9CB-BA0CEE3DD70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C7F1B24-859D-4D35-869A-D9C079BC9517}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D00AC326-0A9F-4BA2-98FC-841FCF1B134A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="151">
   <si>
     <t>PARTIDA_PRESUPUESTARIA</t>
   </si>
@@ -445,13 +445,46 @@
   </si>
   <si>
     <t>TRANSPORTE</t>
+  </si>
+  <si>
+    <t>RUBRO_1</t>
+  </si>
+  <si>
+    <t>RUBRO_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activo </t>
+  </si>
+  <si>
+    <t>Office &amp; Camp</t>
+  </si>
+  <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>RIG SUPPLIES</t>
+  </si>
+  <si>
+    <t>Rig Supplies</t>
+  </si>
+  <si>
+    <t>Other Costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel  &amp; Entertainment </t>
+  </si>
+  <si>
+    <t>Personal Protection Equipments</t>
+  </si>
+  <si>
+    <t>Camp &amp; Catering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -470,6 +503,12 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -479,7 +518,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -680,6 +719,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -687,7 +789,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -704,14 +806,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -722,9 +818,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -734,12 +827,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1057,30 +1179,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9884A49E-A2E9-4497-B62A-DE86A5B60F61}">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="43.85546875" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1090,12 +1220,18 @@
       <c r="C2" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="15" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="E2" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2">
@@ -1104,12 +1240,18 @@
       <c r="C3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="E3" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2">
@@ -1118,12 +1260,18 @@
       <c r="C4" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="E4" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="2">
@@ -1132,12 +1280,18 @@
       <c r="C5" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="E5" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="2">
@@ -1146,12 +1300,18 @@
       <c r="C6" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="E6" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="2">
@@ -1160,12 +1320,18 @@
       <c r="C7" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="E7" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="2">
@@ -1174,12 +1340,18 @@
       <c r="C8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="E8" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="2">
@@ -1188,12 +1360,18 @@
       <c r="C9" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="E9" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="2">
@@ -1202,12 +1380,18 @@
       <c r="C10" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="E10" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="2">
@@ -1216,25 +1400,37 @@
       <c r="C11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="16" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="E11" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="8">
         <v>600155455</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="17" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -1244,12 +1440,18 @@
       <c r="C13" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="15" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="E13" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="2">
@@ -1258,12 +1460,18 @@
       <c r="C14" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="E14" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="2">
@@ -1272,12 +1480,18 @@
       <c r="C15" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="E15" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="2">
@@ -1286,12 +1500,18 @@
       <c r="C16" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="E16" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="2">
@@ -1300,12 +1520,18 @@
       <c r="C17" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="E17" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="2">
@@ -1314,12 +1540,18 @@
       <c r="C18" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="E18" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B19" s="2">
@@ -1328,25 +1560,37 @@
       <c r="C19" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="E19" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>600155511</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="17" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="F20" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1356,12 +1600,18 @@
       <c r="C21" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="15" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="E21" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B22" s="2">
@@ -1370,12 +1620,18 @@
       <c r="C22" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="E22" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="2">
@@ -1384,12 +1640,18 @@
       <c r="C23" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="E23" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B24" s="2">
@@ -1398,12 +1660,18 @@
       <c r="C24" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="E24" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B25" s="2">
@@ -1412,12 +1680,18 @@
       <c r="C25" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="E25" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B26" s="2">
@@ -1426,12 +1700,18 @@
       <c r="C26" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="E26" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B27" s="2">
@@ -1440,12 +1720,18 @@
       <c r="C27" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="E27" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B28" s="2">
@@ -1454,12 +1740,18 @@
       <c r="C28" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+      <c r="E28" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="2">
@@ -1468,12 +1760,18 @@
       <c r="C29" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+      <c r="E29" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B30" s="2">
@@ -1482,12 +1780,18 @@
       <c r="C30" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+      <c r="E30" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B31" s="2">
@@ -1496,12 +1800,18 @@
       <c r="C31" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+      <c r="E31" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B32" s="2">
@@ -1510,12 +1820,18 @@
       <c r="C32" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+      <c r="E32" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B33" s="2">
@@ -1524,12 +1840,18 @@
       <c r="C33" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="E33" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B34" s="2">
@@ -1538,12 +1860,18 @@
       <c r="C34" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
+      <c r="E34" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>37</v>
       </c>
       <c r="B35" s="2">
@@ -1552,12 +1880,18 @@
       <c r="C35" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="E35" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B36" s="2">
@@ -1566,12 +1900,18 @@
       <c r="C36" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
+      <c r="E36" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F36" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B37" s="2">
@@ -1580,12 +1920,18 @@
       <c r="C37" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
+      <c r="E37" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F37" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B38" s="2">
@@ -1594,12 +1940,18 @@
       <c r="C38" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
+      <c r="E38" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B39" s="2">
@@ -1608,12 +1960,18 @@
       <c r="C39" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="7" t="s">
+      <c r="E39" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B40" s="2">
@@ -1622,12 +1980,18 @@
       <c r="C40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D40" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="7" t="s">
+      <c r="E40" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F40" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B41" s="2">
@@ -1636,12 +2000,18 @@
       <c r="C41" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="7" t="s">
+      <c r="E41" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F41" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B42" s="2">
@@ -1650,12 +2020,18 @@
       <c r="C42" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
+      <c r="E42" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F42" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B43" s="2">
@@ -1664,12 +2040,18 @@
       <c r="C43" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D43" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
+      <c r="E43" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F43" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B44" s="2">
@@ -1678,12 +2060,18 @@
       <c r="C44" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="7" t="s">
+      <c r="E44" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F44" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B45" s="2">
@@ -1692,12 +2080,18 @@
       <c r="C45" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="7" t="s">
+      <c r="E45" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F45" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B46" s="2">
@@ -1706,12 +2100,18 @@
       <c r="C46" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="D46" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
+      <c r="E46" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F46" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B47" s="2">
@@ -1720,12 +2120,18 @@
       <c r="C47" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="D47" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="7" t="s">
+      <c r="E47" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F47" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B48" s="2">
@@ -1734,25 +2140,37 @@
       <c r="C48" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D48" s="16" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
+      <c r="E48" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F48" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="10">
+      <c r="B49" s="8">
         <v>500140403</v>
       </c>
-      <c r="C49" s="11" t="s">
+      <c r="C49" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D49" s="12" t="s">
+      <c r="D49" s="17" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="F49" s="24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>52</v>
       </c>
@@ -1762,12 +2180,18 @@
       <c r="C50" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="15" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
+      <c r="E50" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="F50" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B51" s="2">
@@ -1776,12 +2200,18 @@
       <c r="C51" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="D51" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="7" t="s">
+      <c r="E51" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F51" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B52" s="2">
@@ -1790,12 +2220,18 @@
       <c r="C52" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D52" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+      <c r="E52" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F52" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B53" s="2">
@@ -1804,12 +2240,18 @@
       <c r="C53" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D53" s="8" t="s">
+      <c r="D53" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
+      <c r="E53" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F53" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B54" s="2">
@@ -1818,12 +2260,18 @@
       <c r="C54" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D54" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="7" t="s">
+      <c r="E54" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F54" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B55" s="2">
@@ -1832,12 +2280,18 @@
       <c r="C55" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D55" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="7" t="s">
+      <c r="E55" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F55" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B56" s="2">
@@ -1846,12 +2300,18 @@
       <c r="C56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D56" s="8" t="s">
+      <c r="D56" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="7" t="s">
+      <c r="E56" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F56" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
         <v>59</v>
       </c>
       <c r="B57" s="2">
@@ -1860,12 +2320,18 @@
       <c r="C57" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="D57" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="7" t="s">
+      <c r="E57" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F57" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
         <v>60</v>
       </c>
       <c r="B58" s="2">
@@ -1874,12 +2340,18 @@
       <c r="C58" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D58" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="7" t="s">
+      <c r="E58" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F58" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B59" s="2">
@@ -1888,12 +2360,18 @@
       <c r="C59" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="7" t="s">
+      <c r="E59" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F59" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B60" s="2">
@@ -1902,12 +2380,18 @@
       <c r="C60" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D60" s="8" t="s">
+      <c r="D60" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="7" t="s">
+      <c r="E60" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F60" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>63</v>
       </c>
       <c r="B61" s="2">
@@ -1916,12 +2400,18 @@
       <c r="C61" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D61" s="8" t="s">
+      <c r="D61" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="7" t="s">
+      <c r="E61" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F61" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B62" s="2">
@@ -1930,12 +2420,18 @@
       <c r="C62" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D62" s="8" t="s">
+      <c r="D62" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="7" t="s">
+      <c r="E62" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F62" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
         <v>65</v>
       </c>
       <c r="B63" s="2">
@@ -1944,12 +2440,18 @@
       <c r="C63" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D63" s="8" t="s">
+      <c r="D63" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="7" t="s">
+      <c r="E63" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F63" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B64" s="2">
@@ -1958,12 +2460,18 @@
       <c r="C64" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D64" s="8" t="s">
+      <c r="D64" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="7" t="s">
+      <c r="E64" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F64" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
         <v>67</v>
       </c>
       <c r="B65" s="2">
@@ -1972,12 +2480,18 @@
       <c r="C65" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D65" s="8" t="s">
+      <c r="D65" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
+      <c r="E65" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F65" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B66" s="2">
@@ -1986,12 +2500,18 @@
       <c r="C66" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D66" s="8" t="s">
+      <c r="D66" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="7" t="s">
+      <c r="E66" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F66" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
         <v>69</v>
       </c>
       <c r="B67" s="2">
@@ -2000,12 +2520,18 @@
       <c r="C67" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D67" s="8" t="s">
+      <c r="D67" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="7" t="s">
+      <c r="E67" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F67" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="6" t="s">
         <v>70</v>
       </c>
       <c r="B68" s="2">
@@ -2014,25 +2540,37 @@
       <c r="C68" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D68" s="8" t="s">
+      <c r="D68" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="9" t="s">
+      <c r="E68" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F68" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B69" s="10">
+      <c r="B69" s="8">
         <v>500140403</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D69" s="12" t="s">
+      <c r="D69" s="17" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E69" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="F69" s="24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>72</v>
       </c>
@@ -2042,39 +2580,57 @@
       <c r="C70" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D70" s="6" t="s">
+      <c r="D70" s="15" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="9" t="s">
+      <c r="E70" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F70" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B71" s="10">
+      <c r="B71" s="8">
         <v>600155521</v>
       </c>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="D71" s="12" t="s">
+      <c r="D71" s="17" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="13" t="s">
+      <c r="E71" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="F71" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B72" s="14">
+      <c r="B72" s="11">
         <v>600155527</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C72" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="D72" s="16" t="s">
+      <c r="D72" s="18" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="F72" s="29" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>75</v>
       </c>
@@ -2084,12 +2640,18 @@
       <c r="C73" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D73" s="6" t="s">
+      <c r="D73" s="15" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="7" t="s">
+      <c r="E73" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="F73" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
         <v>76</v>
       </c>
       <c r="B74" s="2">
@@ -2098,12 +2660,18 @@
       <c r="C74" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D74" s="8" t="s">
+      <c r="D74" s="16" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="7" t="s">
+      <c r="E74" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="F74" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
         <v>77</v>
       </c>
       <c r="B75" s="2">
@@ -2112,25 +2680,37 @@
       <c r="C75" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D75" s="8" t="s">
+      <c r="D75" s="16" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="9" t="s">
+      <c r="E75" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="F75" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B76" s="10">
+      <c r="B76" s="8">
         <v>500140409</v>
       </c>
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D76" s="12" t="s">
+      <c r="D76" s="17" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="F76" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>79</v>
       </c>
@@ -2140,12 +2720,18 @@
       <c r="C77" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D77" s="6" t="s">
+      <c r="D77" s="15" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="7" t="s">
+      <c r="E77" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F77" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B78" s="2">
@@ -2154,12 +2740,18 @@
       <c r="C78" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="D78" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="7" t="s">
+      <c r="E78" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="F78" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
         <v>81</v>
       </c>
       <c r="B79" s="2">
@@ -2168,12 +2760,18 @@
       <c r="C79" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D79" s="8" t="s">
+      <c r="D79" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="7" t="s">
+      <c r="E79" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F79" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B80" s="2">
@@ -2182,12 +2780,18 @@
       <c r="C80" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D80" s="8" t="s">
+      <c r="D80" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="7" t="s">
+      <c r="E80" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="F80" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
         <v>83</v>
       </c>
       <c r="B81" s="2">
@@ -2196,12 +2800,18 @@
       <c r="C81" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D81" s="8" t="s">
+      <c r="D81" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="7" t="s">
+      <c r="E81" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="F81" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
         <v>84</v>
       </c>
       <c r="B82" s="2">
@@ -2210,12 +2820,18 @@
       <c r="C82" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D82" s="8" t="s">
+      <c r="D82" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="7" t="s">
+      <c r="E82" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F82" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
         <v>85</v>
       </c>
       <c r="B83" s="2">
@@ -2224,12 +2840,18 @@
       <c r="C83" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D83" s="8" t="s">
+      <c r="D83" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="7" t="s">
+      <c r="E83" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F83" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
         <v>86</v>
       </c>
       <c r="B84" s="2">
@@ -2238,12 +2860,18 @@
       <c r="C84" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D84" s="8" t="s">
+      <c r="D84" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="7" t="s">
+      <c r="E84" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F84" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
         <v>87</v>
       </c>
       <c r="B85" s="2">
@@ -2252,12 +2880,18 @@
       <c r="C85" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D85" s="8" t="s">
+      <c r="D85" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="7" t="s">
+      <c r="E85" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F85" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="6" t="s">
         <v>88</v>
       </c>
       <c r="B86" s="2">
@@ -2266,12 +2900,18 @@
       <c r="C86" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D86" s="8" t="s">
+      <c r="D86" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="7" t="s">
+      <c r="E86" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F86" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="6" t="s">
         <v>89</v>
       </c>
       <c r="B87" s="2">
@@ -2280,12 +2920,18 @@
       <c r="C87" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D87" s="8" t="s">
+      <c r="D87" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="7" t="s">
+      <c r="E87" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F87" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
         <v>90</v>
       </c>
       <c r="B88" s="2">
@@ -2294,12 +2940,18 @@
       <c r="C88" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D88" s="8" t="s">
+      <c r="D88" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="7" t="s">
+      <c r="E88" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F88" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="6" t="s">
         <v>91</v>
       </c>
       <c r="B89" s="2">
@@ -2308,12 +2960,18 @@
       <c r="C89" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D89" s="8" t="s">
+      <c r="D89" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="7" t="s">
+      <c r="E89" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F89" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="6" t="s">
         <v>92</v>
       </c>
       <c r="B90" s="2">
@@ -2322,12 +2980,18 @@
       <c r="C90" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D90" s="8" t="s">
+      <c r="D90" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="7" t="s">
+      <c r="E90" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F90" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
         <v>93</v>
       </c>
       <c r="B91" s="2">
@@ -2336,12 +3000,18 @@
       <c r="C91" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D91" s="8" t="s">
+      <c r="D91" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="7" t="s">
+      <c r="E91" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F91" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="6" t="s">
         <v>94</v>
       </c>
       <c r="B92" s="2">
@@ -2350,25 +3020,37 @@
       <c r="C92" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D92" s="8" t="s">
+      <c r="D92" s="16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="9" t="s">
+      <c r="E92" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F92" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B93" s="10">
+      <c r="B93" s="8">
         <v>600155567</v>
       </c>
-      <c r="C93" s="11" t="s">
+      <c r="C93" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D93" s="12" t="s">
+      <c r="D93" s="17" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="F93" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>96</v>
       </c>
@@ -2378,12 +3060,18 @@
       <c r="C94" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D94" s="6" t="s">
+      <c r="D94" s="15" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="7" t="s">
+      <c r="E94" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="F94" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="6" t="s">
         <v>97</v>
       </c>
       <c r="B95" s="2">
@@ -2392,12 +3080,18 @@
       <c r="C95" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D95" s="8" t="s">
+      <c r="D95" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="7" t="s">
+      <c r="E95" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F95" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="6" t="s">
         <v>98</v>
       </c>
       <c r="B96" s="2">
@@ -2406,12 +3100,18 @@
       <c r="C96" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D96" s="8" t="s">
+      <c r="D96" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="7" t="s">
+      <c r="E96" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F96" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="6" t="s">
         <v>99</v>
       </c>
       <c r="B97" s="2">
@@ -2420,12 +3120,18 @@
       <c r="C97" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D97" s="8" t="s">
+      <c r="D97" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="7" t="s">
+      <c r="E97" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F97" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="6" t="s">
         <v>100</v>
       </c>
       <c r="B98" s="2">
@@ -2434,12 +3140,18 @@
       <c r="C98" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D98" s="8" t="s">
+      <c r="D98" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="7" t="s">
+      <c r="E98" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F98" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="6" t="s">
         <v>101</v>
       </c>
       <c r="B99" s="2">
@@ -2448,12 +3160,18 @@
       <c r="C99" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D99" s="8" t="s">
+      <c r="D99" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="7" t="s">
+      <c r="E99" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F99" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
         <v>102</v>
       </c>
       <c r="B100" s="2">
@@ -2462,25 +3180,38 @@
       <c r="C100" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D100" s="8" t="s">
+      <c r="D100" s="16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="9" t="s">
+      <c r="E100" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F100" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B101" s="10">
+      <c r="B101" s="8">
         <v>590130393</v>
       </c>
-      <c r="C101" s="11" t="s">
+      <c r="C101" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="D101" s="12" t="s">
+      <c r="D101" s="17" t="s">
         <v>139</v>
       </c>
+      <c r="E101" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="F101" s="24" t="s">
+        <v>146</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>